<commit_message>
Aplicar formato visual consistente con hojas originales a 'VAN y TIR'
- Hoja 'VAN y TIR':
  · Título (azul, 14pt bold) y subtítulo (azul, 12pt bold)
  · Secciones con fondo naranja (FFC000) igual que 'Detalle Costos'
  · Encabezado de tabla con fondo azul (2E75B6) y texto blanco, alto 32.25
  · Celdas input → fondo amarillo (FFFF00)
  · Celdas fórmula → fondo verde (C6EFCE)
  · Referencias cruzadas → fondo rosa (FFD9E6)
  · Columnas de totales y flujos netos en negrita
  · Separadores visuales cada 6 meses (borde superior)
  · Leyenda al pie idéntica a la de las otras hojas
  · Formato numérico #,##0 para UF, 0.0% para TIR, 0.00% para tasas

- Hoja 'Resultados':
  · Restauradas etiquetas B18/B19 ('Proyecto Puro'/'Proyecto Financiado')
  · TIR anual calculada enlazada en D18/D19 (verde, formato 0.0%),
    siguiendo el mismo patrón de columnas que D6–D16

https://claude.ai/code/session_016WWUYYxtzQy2G7nkCmHbLr
</commit_message>
<xml_diff>
--- a/Evaluacion_i360_Proforma.xlsx
+++ b/Evaluacion_i360_Proforma.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -132,8 +132,45 @@
       <color rgb="FF0000FF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E75B6"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E75B6"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -241,8 +278,33 @@
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -296,12 +358,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border/>
+    <border>
+      <top style="thin"/>
+    </border>
+    <border>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -619,6 +692,72 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="19" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="20" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="20" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="20" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="21" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="21" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="20" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="21" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="21" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="21" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="21" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="19" fillId="21" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="20" fillId="21" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="21" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4365,18 +4504,26 @@
           <t>TIR</t>
         </is>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="135" t="inlineStr">
+        <is>
+          <t>Proyecto Puro</t>
+        </is>
+      </c>
+      <c r="D18" s="136">
         <f>'VAN y TIR'!C69</f>
         <v/>
       </c>
-      <c r="D18" s="133" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="B19" s="4">
+      <c r="B19" s="135" t="inlineStr">
+        <is>
+          <t>Proyecto Financiado</t>
+        </is>
+      </c>
+      <c r="D19" s="136">
         <f>'VAN y TIR'!C70</f>
         <v/>
       </c>
-      <c r="D19" s="133" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -4432,1865 +4579,1915 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ANÁLISIS DE VAN Y TIR — PROYECTO INMOBILIARIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1">
+      <c r="A1" s="137" t="inlineStr">
+        <is>
+          <t>VAN y TIR — Análisis de Rentabilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="138" t="inlineStr">
+        <is>
+          <t>Modelo de Flujos de Caja Mensual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="139" t="inlineStr">
         <is>
           <t>PARÁMETROS DE EVALUACIÓN</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="13.5" customHeight="1">
+      <c r="A4" s="135" t="inlineStr">
         <is>
           <t>Tasa de descuento mensual (input)</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="140" t="n">
         <v>0.01</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="13.5" customHeight="1">
+      <c r="A5" s="135" t="inlineStr">
         <is>
           <t>Tasa de descuento anual equivalente</t>
         </is>
       </c>
-      <c r="C5">
+      <c r="C5" s="141">
         <f>(1+C4)^12-1</f>
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="13.5" customHeight="1">
+      <c r="A6" s="135" t="inlineStr">
         <is>
           <t>Período de análisis (meses)</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="142" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="13.5" customHeight="1">
+      <c r="A7" s="135" t="inlineStr">
         <is>
           <t>Duración de construcción (meses)</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="142" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="13.5" customHeight="1">
+      <c r="A8" s="135" t="inlineStr">
         <is>
           <t>Mes de inicio de pre-ventas (input)</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="142" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="9" ht="13.5" customHeight="1">
+      <c r="A9" s="135" t="inlineStr">
         <is>
           <t>Mes de entrega — recepción final (input)</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="142" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="10" ht="13.5" customHeight="1">
+      <c r="A10" s="135" t="inlineStr">
         <is>
           <t>% Ingresos cobrados en pre-venta (input)</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="143" t="n">
         <v>0.3</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="13.5" customHeight="1">
+      <c r="A11" s="135" t="inlineStr">
         <is>
           <t>Mes inicio — Proyectos, Permisos y Empalmes (input)</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="C11" s="142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="13.5" customHeight="1">
+      <c r="A12" s="135" t="inlineStr">
         <is>
           <t>Mes término — Proyectos, Permisos y Empalmes (input)</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="142" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="13" ht="6" customHeight="1"/>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="139" t="inlineStr">
         <is>
           <t>DATOS DEL PROYECTO (referencias a otras hojas)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="15" ht="13.5" customHeight="1">
+      <c r="A15" s="135" t="inlineStr">
         <is>
           <t>Ingresos Totales</t>
         </is>
       </c>
-      <c r="C15">
+      <c r="C15" s="144">
         <f>'Superficies y Valores'!R22</f>
         <v/>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="135" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="16" ht="13.5" customHeight="1">
+      <c r="A16" s="135" t="inlineStr">
         <is>
           <t>Costo Terreno</t>
         </is>
       </c>
-      <c r="C16">
+      <c r="C16" s="144">
         <f>'Detalle Costos'!E4</f>
         <v/>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="135" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="17" ht="13.5" customHeight="1">
+      <c r="A17" s="135" t="inlineStr">
         <is>
           <t>Costo Construcción sin IVA</t>
         </is>
       </c>
-      <c r="C17">
+      <c r="C17" s="144">
         <f>'Detalle Costos'!E10</f>
         <v/>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="135" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="18" ht="13.5" customHeight="1">
+      <c r="A18" s="135" t="inlineStr">
         <is>
           <t>Costos Proyectos, Permisos y Empalmes</t>
         </is>
       </c>
-      <c r="C18">
+      <c r="C18" s="144">
         <f>'Detalle Costos'!E46</f>
         <v/>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="135" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="19" ht="13.5" customHeight="1">
+      <c r="A19" s="135" t="inlineStr">
         <is>
           <t>Costos Adm., Gestión y Ventas</t>
         </is>
       </c>
-      <c r="C19">
+      <c r="C19" s="144">
         <f>'Detalle Costos'!E55</f>
         <v/>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="135" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="20" ht="13.5" customHeight="1">
+      <c r="A20" s="135" t="inlineStr">
         <is>
           <t>Costo Financiero</t>
         </is>
       </c>
-      <c r="C20">
+      <c r="C20" s="144">
         <f>'Detalle Costos'!E67</f>
         <v/>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="135" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="21" ht="13.5" customHeight="1">
+      <c r="A21" s="135" t="inlineStr">
         <is>
           <t>IVA a Pagar</t>
         </is>
       </c>
-      <c r="C21">
+      <c r="C21" s="144">
         <f>'Detalle Costos'!E69</f>
         <v/>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="135" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="22" ht="13.5" customHeight="1">
+      <c r="A22" s="135" t="inlineStr">
         <is>
           <t>Costo Total Proyecto Puro (sin IVA a pagar)</t>
         </is>
       </c>
-      <c r="C22">
+      <c r="C22" s="144">
         <f>'Detalle Costos'!E68</f>
         <v/>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="135" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="23" ht="13.5" customHeight="1">
+      <c r="A23" s="135" t="inlineStr">
         <is>
           <t>Costo Total Proyecto Financiado (con IVA a pagar)</t>
         </is>
       </c>
-      <c r="C23">
+      <c r="C23" s="144">
         <f>'Detalle Costos'!E70</f>
         <v/>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="135" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="24" ht="6" customHeight="1"/>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="139" t="inlineStr">
         <is>
           <t>SUPUESTOS DE DISTRIBUCIÓN TEMPORAL</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="26" ht="13" customHeight="1">
+      <c r="A26" s="145" t="inlineStr">
         <is>
           <t>• Terreno: 100 % en el mes 0</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="145" t="inlineStr">
         <is>
           <t>• Construcción sin IVA: distribuido uniformemente en los meses 1 a C7</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="28" ht="13" customHeight="1">
+      <c r="A28" s="145" t="inlineStr">
         <is>
           <t>• Proyectos, Permisos y Empalmes: distribuido uniformemente en los meses C11 a C12 (ajustable)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="29" ht="13" customHeight="1">
+      <c r="A29" s="145" t="inlineStr">
         <is>
           <t>• Adm., Gestión y Ventas: distribuido uniformemente desde el mes C8 hasta el mes C9</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="30" ht="13" customHeight="1">
+      <c r="A30" s="145" t="inlineStr">
         <is>
           <t>• Costo Financiero e IVA a Pagar: íntegramente en el mes de entrega (C9)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="31" ht="13" customHeight="1">
+      <c r="A31" s="145" t="inlineStr">
         <is>
           <t>• Ingresos Pre-venta (C10 = 30 %): distribuidos uniformemente desde el mes C8 hasta el mes C9-1</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="32" ht="13" customHeight="1">
+      <c r="A32" s="145" t="inlineStr">
         <is>
           <t>• Ingresos de Entrega (1-C10 = 70 %): íntegramente en el mes de entrega (C9)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="139" t="inlineStr">
         <is>
           <t>TABLA DE FLUJOS DE CAJA (montos en UF)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="34" ht="32.25" customHeight="1">
+      <c r="A34" s="146" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="146" t="inlineStr">
         <is>
           <t>Ing. Pre-venta</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="146" t="inlineStr">
         <is>
           <t>Ing. Entrega</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="146" t="inlineStr">
         <is>
           <t>Total Ingresos</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="146" t="inlineStr">
         <is>
           <t>Terreno</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="146" t="inlineStr">
         <is>
           <t>Construcción</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="146" t="inlineStr">
         <is>
           <t>Proy. y Permisos</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" s="146" t="inlineStr">
         <is>
           <t>Adm. y Ventas</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="146" t="inlineStr">
         <is>
           <t>Costo Financiero</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="146" t="inlineStr">
         <is>
           <t>Total Egresos Puro</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K34" s="146" t="inlineStr">
         <is>
           <t>Flujo Neto Puro</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L34" s="146" t="inlineStr">
         <is>
           <t>IVA a Pagar</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M34" s="146" t="inlineStr">
         <is>
           <t>Total Egresos Financiado</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="N34" s="146" t="inlineStr">
         <is>
           <t>Flujo Neto Financiado</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>0</v>
-      </c>
-      <c r="B35">
+    <row r="35" ht="13" customHeight="1">
+      <c r="A35" s="147" t="n">
+        <v>0</v>
+      </c>
+      <c r="B35" s="148">
         <f>IF(AND($A35&gt;=$C$8,$A35&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C35">
+      <c r="C35" s="148">
         <f>IF($A35=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D35">
+      <c r="D35" s="149">
         <f>B35+C35</f>
         <v/>
       </c>
-      <c r="E35">
+      <c r="E35" s="148">
         <f>IF($A35=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F35">
+      <c r="F35" s="148">
         <f>IF(AND($A35&gt;=1,$A35&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G35">
+      <c r="G35" s="148">
         <f>IF(AND($A35&gt;=$C$11,$A35&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H35">
+      <c r="H35" s="148">
         <f>IF(AND($A35&gt;=$C$8,$A35&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I35">
+      <c r="I35" s="148">
         <f>IF($A35=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J35">
+      <c r="J35" s="149">
         <f>E35+F35+G35+H35+I35</f>
         <v/>
       </c>
-      <c r="K35">
+      <c r="K35" s="149">
         <f>D35-J35</f>
         <v/>
       </c>
-      <c r="L35">
+      <c r="L35" s="148">
         <f>IF($A35=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M35">
+      <c r="M35" s="149">
         <f>J35+L35</f>
         <v/>
       </c>
-      <c r="N35">
+      <c r="N35" s="149">
         <f>D35-M35</f>
         <v/>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="n">
+    <row r="36" ht="13" customHeight="1">
+      <c r="A36" s="147" t="n">
         <v>1</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="148">
         <f>IF(AND($A36&gt;=$C$8,$A36&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C36">
+      <c r="C36" s="148">
         <f>IF($A36=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D36">
+      <c r="D36" s="149">
         <f>B36+C36</f>
         <v/>
       </c>
-      <c r="E36">
+      <c r="E36" s="148">
         <f>IF($A36=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F36">
+      <c r="F36" s="148">
         <f>IF(AND($A36&gt;=1,$A36&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G36">
+      <c r="G36" s="148">
         <f>IF(AND($A36&gt;=$C$11,$A36&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H36">
+      <c r="H36" s="148">
         <f>IF(AND($A36&gt;=$C$8,$A36&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I36">
+      <c r="I36" s="148">
         <f>IF($A36=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J36">
+      <c r="J36" s="149">
         <f>E36+F36+G36+H36+I36</f>
         <v/>
       </c>
-      <c r="K36">
+      <c r="K36" s="149">
         <f>D36-J36</f>
         <v/>
       </c>
-      <c r="L36">
+      <c r="L36" s="148">
         <f>IF($A36=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M36">
+      <c r="M36" s="149">
         <f>J36+L36</f>
         <v/>
       </c>
-      <c r="N36">
+      <c r="N36" s="149">
         <f>D36-M36</f>
         <v/>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="n">
+    <row r="37" ht="13" customHeight="1">
+      <c r="A37" s="147" t="n">
         <v>2</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="148">
         <f>IF(AND($A37&gt;=$C$8,$A37&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C37">
+      <c r="C37" s="148">
         <f>IF($A37=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D37">
+      <c r="D37" s="149">
         <f>B37+C37</f>
         <v/>
       </c>
-      <c r="E37">
+      <c r="E37" s="148">
         <f>IF($A37=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F37">
+      <c r="F37" s="148">
         <f>IF(AND($A37&gt;=1,$A37&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G37">
+      <c r="G37" s="148">
         <f>IF(AND($A37&gt;=$C$11,$A37&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H37">
+      <c r="H37" s="148">
         <f>IF(AND($A37&gt;=$C$8,$A37&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I37">
+      <c r="I37" s="148">
         <f>IF($A37=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J37">
+      <c r="J37" s="149">
         <f>E37+F37+G37+H37+I37</f>
         <v/>
       </c>
-      <c r="K37">
+      <c r="K37" s="149">
         <f>D37-J37</f>
         <v/>
       </c>
-      <c r="L37">
+      <c r="L37" s="148">
         <f>IF($A37=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M37">
+      <c r="M37" s="149">
         <f>J37+L37</f>
         <v/>
       </c>
-      <c r="N37">
+      <c r="N37" s="149">
         <f>D37-M37</f>
         <v/>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="n">
+    <row r="38" ht="13" customHeight="1">
+      <c r="A38" s="147" t="n">
         <v>3</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="148">
         <f>IF(AND($A38&gt;=$C$8,$A38&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C38">
+      <c r="C38" s="148">
         <f>IF($A38=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D38">
+      <c r="D38" s="149">
         <f>B38+C38</f>
         <v/>
       </c>
-      <c r="E38">
+      <c r="E38" s="148">
         <f>IF($A38=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F38">
+      <c r="F38" s="148">
         <f>IF(AND($A38&gt;=1,$A38&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G38">
+      <c r="G38" s="148">
         <f>IF(AND($A38&gt;=$C$11,$A38&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H38">
+      <c r="H38" s="148">
         <f>IF(AND($A38&gt;=$C$8,$A38&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I38">
+      <c r="I38" s="148">
         <f>IF($A38=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J38">
+      <c r="J38" s="149">
         <f>E38+F38+G38+H38+I38</f>
         <v/>
       </c>
-      <c r="K38">
+      <c r="K38" s="149">
         <f>D38-J38</f>
         <v/>
       </c>
-      <c r="L38">
+      <c r="L38" s="148">
         <f>IF($A38=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M38">
+      <c r="M38" s="149">
         <f>J38+L38</f>
         <v/>
       </c>
-      <c r="N38">
+      <c r="N38" s="149">
         <f>D38-M38</f>
         <v/>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="n">
+    <row r="39" ht="13" customHeight="1">
+      <c r="A39" s="147" t="n">
         <v>4</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="148">
         <f>IF(AND($A39&gt;=$C$8,$A39&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C39">
+      <c r="C39" s="148">
         <f>IF($A39=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D39">
+      <c r="D39" s="149">
         <f>B39+C39</f>
         <v/>
       </c>
-      <c r="E39">
+      <c r="E39" s="148">
         <f>IF($A39=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F39">
+      <c r="F39" s="148">
         <f>IF(AND($A39&gt;=1,$A39&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G39">
+      <c r="G39" s="148">
         <f>IF(AND($A39&gt;=$C$11,$A39&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H39">
+      <c r="H39" s="148">
         <f>IF(AND($A39&gt;=$C$8,$A39&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I39">
+      <c r="I39" s="148">
         <f>IF($A39=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J39">
+      <c r="J39" s="149">
         <f>E39+F39+G39+H39+I39</f>
         <v/>
       </c>
-      <c r="K39">
+      <c r="K39" s="149">
         <f>D39-J39</f>
         <v/>
       </c>
-      <c r="L39">
+      <c r="L39" s="148">
         <f>IF($A39=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M39">
+      <c r="M39" s="149">
         <f>J39+L39</f>
         <v/>
       </c>
-      <c r="N39">
+      <c r="N39" s="149">
         <f>D39-M39</f>
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="n">
+    <row r="40" ht="13" customHeight="1">
+      <c r="A40" s="147" t="n">
         <v>5</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="148">
         <f>IF(AND($A40&gt;=$C$8,$A40&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C40">
+      <c r="C40" s="148">
         <f>IF($A40=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D40">
+      <c r="D40" s="149">
         <f>B40+C40</f>
         <v/>
       </c>
-      <c r="E40">
+      <c r="E40" s="148">
         <f>IF($A40=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F40">
+      <c r="F40" s="148">
         <f>IF(AND($A40&gt;=1,$A40&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G40">
+      <c r="G40" s="148">
         <f>IF(AND($A40&gt;=$C$11,$A40&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H40">
+      <c r="H40" s="148">
         <f>IF(AND($A40&gt;=$C$8,$A40&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I40">
+      <c r="I40" s="148">
         <f>IF($A40=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J40">
+      <c r="J40" s="149">
         <f>E40+F40+G40+H40+I40</f>
         <v/>
       </c>
-      <c r="K40">
+      <c r="K40" s="149">
         <f>D40-J40</f>
         <v/>
       </c>
-      <c r="L40">
+      <c r="L40" s="148">
         <f>IF($A40=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M40">
+      <c r="M40" s="149">
         <f>J40+L40</f>
         <v/>
       </c>
-      <c r="N40">
+      <c r="N40" s="149">
         <f>D40-M40</f>
         <v/>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="n">
+    <row r="41" ht="13" customHeight="1">
+      <c r="A41" s="150" t="n">
         <v>6</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="151">
         <f>IF(AND($A41&gt;=$C$8,$A41&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C41">
+      <c r="C41" s="151">
         <f>IF($A41=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D41">
+      <c r="D41" s="152">
         <f>B41+C41</f>
         <v/>
       </c>
-      <c r="E41">
+      <c r="E41" s="151">
         <f>IF($A41=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F41">
+      <c r="F41" s="151">
         <f>IF(AND($A41&gt;=1,$A41&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G41">
+      <c r="G41" s="151">
         <f>IF(AND($A41&gt;=$C$11,$A41&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H41">
+      <c r="H41" s="151">
         <f>IF(AND($A41&gt;=$C$8,$A41&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I41">
+      <c r="I41" s="151">
         <f>IF($A41=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J41">
+      <c r="J41" s="152">
         <f>E41+F41+G41+H41+I41</f>
         <v/>
       </c>
-      <c r="K41">
+      <c r="K41" s="152">
         <f>D41-J41</f>
         <v/>
       </c>
-      <c r="L41">
+      <c r="L41" s="151">
         <f>IF($A41=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M41">
+      <c r="M41" s="152">
         <f>J41+L41</f>
         <v/>
       </c>
-      <c r="N41">
+      <c r="N41" s="152">
         <f>D41-M41</f>
         <v/>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="n">
+    <row r="42" ht="13" customHeight="1">
+      <c r="A42" s="147" t="n">
         <v>7</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="148">
         <f>IF(AND($A42&gt;=$C$8,$A42&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C42">
+      <c r="C42" s="148">
         <f>IF($A42=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D42">
+      <c r="D42" s="149">
         <f>B42+C42</f>
         <v/>
       </c>
-      <c r="E42">
+      <c r="E42" s="148">
         <f>IF($A42=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F42">
+      <c r="F42" s="148">
         <f>IF(AND($A42&gt;=1,$A42&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G42">
+      <c r="G42" s="148">
         <f>IF(AND($A42&gt;=$C$11,$A42&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H42">
+      <c r="H42" s="148">
         <f>IF(AND($A42&gt;=$C$8,$A42&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I42">
+      <c r="I42" s="148">
         <f>IF($A42=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J42">
+      <c r="J42" s="149">
         <f>E42+F42+G42+H42+I42</f>
         <v/>
       </c>
-      <c r="K42">
+      <c r="K42" s="149">
         <f>D42-J42</f>
         <v/>
       </c>
-      <c r="L42">
+      <c r="L42" s="148">
         <f>IF($A42=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M42">
+      <c r="M42" s="149">
         <f>J42+L42</f>
         <v/>
       </c>
-      <c r="N42">
+      <c r="N42" s="149">
         <f>D42-M42</f>
         <v/>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="n">
+    <row r="43" ht="13" customHeight="1">
+      <c r="A43" s="147" t="n">
         <v>8</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="148">
         <f>IF(AND($A43&gt;=$C$8,$A43&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C43">
+      <c r="C43" s="148">
         <f>IF($A43=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D43">
+      <c r="D43" s="149">
         <f>B43+C43</f>
         <v/>
       </c>
-      <c r="E43">
+      <c r="E43" s="148">
         <f>IF($A43=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F43">
+      <c r="F43" s="148">
         <f>IF(AND($A43&gt;=1,$A43&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G43">
+      <c r="G43" s="148">
         <f>IF(AND($A43&gt;=$C$11,$A43&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H43">
+      <c r="H43" s="148">
         <f>IF(AND($A43&gt;=$C$8,$A43&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I43">
+      <c r="I43" s="148">
         <f>IF($A43=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J43">
+      <c r="J43" s="149">
         <f>E43+F43+G43+H43+I43</f>
         <v/>
       </c>
-      <c r="K43">
+      <c r="K43" s="149">
         <f>D43-J43</f>
         <v/>
       </c>
-      <c r="L43">
+      <c r="L43" s="148">
         <f>IF($A43=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M43">
+      <c r="M43" s="149">
         <f>J43+L43</f>
         <v/>
       </c>
-      <c r="N43">
+      <c r="N43" s="149">
         <f>D43-M43</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="n">
+    <row r="44" ht="13" customHeight="1">
+      <c r="A44" s="147" t="n">
         <v>9</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="148">
         <f>IF(AND($A44&gt;=$C$8,$A44&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C44">
+      <c r="C44" s="148">
         <f>IF($A44=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D44">
+      <c r="D44" s="149">
         <f>B44+C44</f>
         <v/>
       </c>
-      <c r="E44">
+      <c r="E44" s="148">
         <f>IF($A44=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F44">
+      <c r="F44" s="148">
         <f>IF(AND($A44&gt;=1,$A44&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G44">
+      <c r="G44" s="148">
         <f>IF(AND($A44&gt;=$C$11,$A44&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H44">
+      <c r="H44" s="148">
         <f>IF(AND($A44&gt;=$C$8,$A44&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I44">
+      <c r="I44" s="148">
         <f>IF($A44=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J44">
+      <c r="J44" s="149">
         <f>E44+F44+G44+H44+I44</f>
         <v/>
       </c>
-      <c r="K44">
+      <c r="K44" s="149">
         <f>D44-J44</f>
         <v/>
       </c>
-      <c r="L44">
+      <c r="L44" s="148">
         <f>IF($A44=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M44">
+      <c r="M44" s="149">
         <f>J44+L44</f>
         <v/>
       </c>
-      <c r="N44">
+      <c r="N44" s="149">
         <f>D44-M44</f>
         <v/>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="n">
+    <row r="45" ht="13" customHeight="1">
+      <c r="A45" s="147" t="n">
         <v>10</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="148">
         <f>IF(AND($A45&gt;=$C$8,$A45&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C45">
+      <c r="C45" s="148">
         <f>IF($A45=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D45">
+      <c r="D45" s="149">
         <f>B45+C45</f>
         <v/>
       </c>
-      <c r="E45">
+      <c r="E45" s="148">
         <f>IF($A45=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F45">
+      <c r="F45" s="148">
         <f>IF(AND($A45&gt;=1,$A45&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G45">
+      <c r="G45" s="148">
         <f>IF(AND($A45&gt;=$C$11,$A45&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H45">
+      <c r="H45" s="148">
         <f>IF(AND($A45&gt;=$C$8,$A45&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I45">
+      <c r="I45" s="148">
         <f>IF($A45=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J45">
+      <c r="J45" s="149">
         <f>E45+F45+G45+H45+I45</f>
         <v/>
       </c>
-      <c r="K45">
+      <c r="K45" s="149">
         <f>D45-J45</f>
         <v/>
       </c>
-      <c r="L45">
+      <c r="L45" s="148">
         <f>IF($A45=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M45">
+      <c r="M45" s="149">
         <f>J45+L45</f>
         <v/>
       </c>
-      <c r="N45">
+      <c r="N45" s="149">
         <f>D45-M45</f>
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="n">
+    <row r="46" ht="13" customHeight="1">
+      <c r="A46" s="147" t="n">
         <v>11</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="148">
         <f>IF(AND($A46&gt;=$C$8,$A46&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C46">
+      <c r="C46" s="148">
         <f>IF($A46=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D46">
+      <c r="D46" s="149">
         <f>B46+C46</f>
         <v/>
       </c>
-      <c r="E46">
+      <c r="E46" s="148">
         <f>IF($A46=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F46">
+      <c r="F46" s="148">
         <f>IF(AND($A46&gt;=1,$A46&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G46">
+      <c r="G46" s="148">
         <f>IF(AND($A46&gt;=$C$11,$A46&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H46">
+      <c r="H46" s="148">
         <f>IF(AND($A46&gt;=$C$8,$A46&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I46">
+      <c r="I46" s="148">
         <f>IF($A46=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J46">
+      <c r="J46" s="149">
         <f>E46+F46+G46+H46+I46</f>
         <v/>
       </c>
-      <c r="K46">
+      <c r="K46" s="149">
         <f>D46-J46</f>
         <v/>
       </c>
-      <c r="L46">
+      <c r="L46" s="148">
         <f>IF($A46=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M46">
+      <c r="M46" s="149">
         <f>J46+L46</f>
         <v/>
       </c>
-      <c r="N46">
+      <c r="N46" s="149">
         <f>D46-M46</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="n">
+    <row r="47" ht="13" customHeight="1">
+      <c r="A47" s="150" t="n">
         <v>12</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="151">
         <f>IF(AND($A47&gt;=$C$8,$A47&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C47">
+      <c r="C47" s="151">
         <f>IF($A47=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D47">
+      <c r="D47" s="152">
         <f>B47+C47</f>
         <v/>
       </c>
-      <c r="E47">
+      <c r="E47" s="151">
         <f>IF($A47=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F47">
+      <c r="F47" s="151">
         <f>IF(AND($A47&gt;=1,$A47&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G47">
+      <c r="G47" s="151">
         <f>IF(AND($A47&gt;=$C$11,$A47&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H47">
+      <c r="H47" s="151">
         <f>IF(AND($A47&gt;=$C$8,$A47&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I47">
+      <c r="I47" s="151">
         <f>IF($A47=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J47">
+      <c r="J47" s="152">
         <f>E47+F47+G47+H47+I47</f>
         <v/>
       </c>
-      <c r="K47">
+      <c r="K47" s="152">
         <f>D47-J47</f>
         <v/>
       </c>
-      <c r="L47">
+      <c r="L47" s="151">
         <f>IF($A47=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M47">
+      <c r="M47" s="152">
         <f>J47+L47</f>
         <v/>
       </c>
-      <c r="N47">
+      <c r="N47" s="152">
         <f>D47-M47</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="n">
+    <row r="48" ht="13" customHeight="1">
+      <c r="A48" s="147" t="n">
         <v>13</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="148">
         <f>IF(AND($A48&gt;=$C$8,$A48&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C48">
+      <c r="C48" s="148">
         <f>IF($A48=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D48">
+      <c r="D48" s="149">
         <f>B48+C48</f>
         <v/>
       </c>
-      <c r="E48">
+      <c r="E48" s="148">
         <f>IF($A48=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F48">
+      <c r="F48" s="148">
         <f>IF(AND($A48&gt;=1,$A48&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G48">
+      <c r="G48" s="148">
         <f>IF(AND($A48&gt;=$C$11,$A48&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H48">
+      <c r="H48" s="148">
         <f>IF(AND($A48&gt;=$C$8,$A48&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I48">
+      <c r="I48" s="148">
         <f>IF($A48=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J48">
+      <c r="J48" s="149">
         <f>E48+F48+G48+H48+I48</f>
         <v/>
       </c>
-      <c r="K48">
+      <c r="K48" s="149">
         <f>D48-J48</f>
         <v/>
       </c>
-      <c r="L48">
+      <c r="L48" s="148">
         <f>IF($A48=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M48">
+      <c r="M48" s="149">
         <f>J48+L48</f>
         <v/>
       </c>
-      <c r="N48">
+      <c r="N48" s="149">
         <f>D48-M48</f>
         <v/>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="n">
+    <row r="49" ht="13" customHeight="1">
+      <c r="A49" s="147" t="n">
         <v>14</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="148">
         <f>IF(AND($A49&gt;=$C$8,$A49&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C49">
+      <c r="C49" s="148">
         <f>IF($A49=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D49">
+      <c r="D49" s="149">
         <f>B49+C49</f>
         <v/>
       </c>
-      <c r="E49">
+      <c r="E49" s="148">
         <f>IF($A49=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F49">
+      <c r="F49" s="148">
         <f>IF(AND($A49&gt;=1,$A49&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G49">
+      <c r="G49" s="148">
         <f>IF(AND($A49&gt;=$C$11,$A49&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H49">
+      <c r="H49" s="148">
         <f>IF(AND($A49&gt;=$C$8,$A49&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I49">
+      <c r="I49" s="148">
         <f>IF($A49=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J49">
+      <c r="J49" s="149">
         <f>E49+F49+G49+H49+I49</f>
         <v/>
       </c>
-      <c r="K49">
+      <c r="K49" s="149">
         <f>D49-J49</f>
         <v/>
       </c>
-      <c r="L49">
+      <c r="L49" s="148">
         <f>IF($A49=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M49">
+      <c r="M49" s="149">
         <f>J49+L49</f>
         <v/>
       </c>
-      <c r="N49">
+      <c r="N49" s="149">
         <f>D49-M49</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="n">
+    <row r="50" ht="13" customHeight="1">
+      <c r="A50" s="147" t="n">
         <v>15</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="148">
         <f>IF(AND($A50&gt;=$C$8,$A50&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C50">
+      <c r="C50" s="148">
         <f>IF($A50=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D50">
+      <c r="D50" s="149">
         <f>B50+C50</f>
         <v/>
       </c>
-      <c r="E50">
+      <c r="E50" s="148">
         <f>IF($A50=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F50">
+      <c r="F50" s="148">
         <f>IF(AND($A50&gt;=1,$A50&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G50">
+      <c r="G50" s="148">
         <f>IF(AND($A50&gt;=$C$11,$A50&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H50">
+      <c r="H50" s="148">
         <f>IF(AND($A50&gt;=$C$8,$A50&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I50">
+      <c r="I50" s="148">
         <f>IF($A50=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J50">
+      <c r="J50" s="149">
         <f>E50+F50+G50+H50+I50</f>
         <v/>
       </c>
-      <c r="K50">
+      <c r="K50" s="149">
         <f>D50-J50</f>
         <v/>
       </c>
-      <c r="L50">
+      <c r="L50" s="148">
         <f>IF($A50=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M50">
+      <c r="M50" s="149">
         <f>J50+L50</f>
         <v/>
       </c>
-      <c r="N50">
+      <c r="N50" s="149">
         <f>D50-M50</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="n">
+    <row r="51" ht="13" customHeight="1">
+      <c r="A51" s="147" t="n">
         <v>16</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="148">
         <f>IF(AND($A51&gt;=$C$8,$A51&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C51">
+      <c r="C51" s="148">
         <f>IF($A51=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D51">
+      <c r="D51" s="149">
         <f>B51+C51</f>
         <v/>
       </c>
-      <c r="E51">
+      <c r="E51" s="148">
         <f>IF($A51=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F51">
+      <c r="F51" s="148">
         <f>IF(AND($A51&gt;=1,$A51&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G51">
+      <c r="G51" s="148">
         <f>IF(AND($A51&gt;=$C$11,$A51&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H51">
+      <c r="H51" s="148">
         <f>IF(AND($A51&gt;=$C$8,$A51&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I51">
+      <c r="I51" s="148">
         <f>IF($A51=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J51">
+      <c r="J51" s="149">
         <f>E51+F51+G51+H51+I51</f>
         <v/>
       </c>
-      <c r="K51">
+      <c r="K51" s="149">
         <f>D51-J51</f>
         <v/>
       </c>
-      <c r="L51">
+      <c r="L51" s="148">
         <f>IF($A51=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M51">
+      <c r="M51" s="149">
         <f>J51+L51</f>
         <v/>
       </c>
-      <c r="N51">
+      <c r="N51" s="149">
         <f>D51-M51</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="n">
+    <row r="52" ht="13" customHeight="1">
+      <c r="A52" s="147" t="n">
         <v>17</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="148">
         <f>IF(AND($A52&gt;=$C$8,$A52&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C52">
+      <c r="C52" s="148">
         <f>IF($A52=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D52">
+      <c r="D52" s="149">
         <f>B52+C52</f>
         <v/>
       </c>
-      <c r="E52">
+      <c r="E52" s="148">
         <f>IF($A52=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F52">
+      <c r="F52" s="148">
         <f>IF(AND($A52&gt;=1,$A52&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G52">
+      <c r="G52" s="148">
         <f>IF(AND($A52&gt;=$C$11,$A52&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H52">
+      <c r="H52" s="148">
         <f>IF(AND($A52&gt;=$C$8,$A52&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I52">
+      <c r="I52" s="148">
         <f>IF($A52=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J52">
+      <c r="J52" s="149">
         <f>E52+F52+G52+H52+I52</f>
         <v/>
       </c>
-      <c r="K52">
+      <c r="K52" s="149">
         <f>D52-J52</f>
         <v/>
       </c>
-      <c r="L52">
+      <c r="L52" s="148">
         <f>IF($A52=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M52">
+      <c r="M52" s="149">
         <f>J52+L52</f>
         <v/>
       </c>
-      <c r="N52">
+      <c r="N52" s="149">
         <f>D52-M52</f>
         <v/>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="n">
+    <row r="53" ht="13" customHeight="1">
+      <c r="A53" s="150" t="n">
         <v>18</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="151">
         <f>IF(AND($A53&gt;=$C$8,$A53&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C53">
+      <c r="C53" s="151">
         <f>IF($A53=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D53">
+      <c r="D53" s="152">
         <f>B53+C53</f>
         <v/>
       </c>
-      <c r="E53">
+      <c r="E53" s="151">
         <f>IF($A53=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F53">
+      <c r="F53" s="151">
         <f>IF(AND($A53&gt;=1,$A53&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G53">
+      <c r="G53" s="151">
         <f>IF(AND($A53&gt;=$C$11,$A53&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H53">
+      <c r="H53" s="151">
         <f>IF(AND($A53&gt;=$C$8,$A53&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I53">
+      <c r="I53" s="151">
         <f>IF($A53=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J53">
+      <c r="J53" s="152">
         <f>E53+F53+G53+H53+I53</f>
         <v/>
       </c>
-      <c r="K53">
+      <c r="K53" s="152">
         <f>D53-J53</f>
         <v/>
       </c>
-      <c r="L53">
+      <c r="L53" s="151">
         <f>IF($A53=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M53">
+      <c r="M53" s="152">
         <f>J53+L53</f>
         <v/>
       </c>
-      <c r="N53">
+      <c r="N53" s="152">
         <f>D53-M53</f>
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="n">
+    <row r="54" ht="13" customHeight="1">
+      <c r="A54" s="147" t="n">
         <v>19</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="148">
         <f>IF(AND($A54&gt;=$C$8,$A54&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C54">
+      <c r="C54" s="148">
         <f>IF($A54=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D54">
+      <c r="D54" s="149">
         <f>B54+C54</f>
         <v/>
       </c>
-      <c r="E54">
+      <c r="E54" s="148">
         <f>IF($A54=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F54">
+      <c r="F54" s="148">
         <f>IF(AND($A54&gt;=1,$A54&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G54">
+      <c r="G54" s="148">
         <f>IF(AND($A54&gt;=$C$11,$A54&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H54">
+      <c r="H54" s="148">
         <f>IF(AND($A54&gt;=$C$8,$A54&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I54">
+      <c r="I54" s="148">
         <f>IF($A54=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J54">
+      <c r="J54" s="149">
         <f>E54+F54+G54+H54+I54</f>
         <v/>
       </c>
-      <c r="K54">
+      <c r="K54" s="149">
         <f>D54-J54</f>
         <v/>
       </c>
-      <c r="L54">
+      <c r="L54" s="148">
         <f>IF($A54=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M54">
+      <c r="M54" s="149">
         <f>J54+L54</f>
         <v/>
       </c>
-      <c r="N54">
+      <c r="N54" s="149">
         <f>D54-M54</f>
         <v/>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="n">
+    <row r="55" ht="13" customHeight="1">
+      <c r="A55" s="147" t="n">
         <v>20</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="148">
         <f>IF(AND($A55&gt;=$C$8,$A55&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C55">
+      <c r="C55" s="148">
         <f>IF($A55=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D55">
+      <c r="D55" s="149">
         <f>B55+C55</f>
         <v/>
       </c>
-      <c r="E55">
+      <c r="E55" s="148">
         <f>IF($A55=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F55">
+      <c r="F55" s="148">
         <f>IF(AND($A55&gt;=1,$A55&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G55">
+      <c r="G55" s="148">
         <f>IF(AND($A55&gt;=$C$11,$A55&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H55">
+      <c r="H55" s="148">
         <f>IF(AND($A55&gt;=$C$8,$A55&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I55">
+      <c r="I55" s="148">
         <f>IF($A55=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J55">
+      <c r="J55" s="149">
         <f>E55+F55+G55+H55+I55</f>
         <v/>
       </c>
-      <c r="K55">
+      <c r="K55" s="149">
         <f>D55-J55</f>
         <v/>
       </c>
-      <c r="L55">
+      <c r="L55" s="148">
         <f>IF($A55=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M55">
+      <c r="M55" s="149">
         <f>J55+L55</f>
         <v/>
       </c>
-      <c r="N55">
+      <c r="N55" s="149">
         <f>D55-M55</f>
         <v/>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="n">
+    <row r="56" ht="13" customHeight="1">
+      <c r="A56" s="147" t="n">
         <v>21</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="148">
         <f>IF(AND($A56&gt;=$C$8,$A56&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C56">
+      <c r="C56" s="148">
         <f>IF($A56=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D56">
+      <c r="D56" s="149">
         <f>B56+C56</f>
         <v/>
       </c>
-      <c r="E56">
+      <c r="E56" s="148">
         <f>IF($A56=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F56">
+      <c r="F56" s="148">
         <f>IF(AND($A56&gt;=1,$A56&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G56">
+      <c r="G56" s="148">
         <f>IF(AND($A56&gt;=$C$11,$A56&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H56">
+      <c r="H56" s="148">
         <f>IF(AND($A56&gt;=$C$8,$A56&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I56">
+      <c r="I56" s="148">
         <f>IF($A56=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J56">
+      <c r="J56" s="149">
         <f>E56+F56+G56+H56+I56</f>
         <v/>
       </c>
-      <c r="K56">
+      <c r="K56" s="149">
         <f>D56-J56</f>
         <v/>
       </c>
-      <c r="L56">
+      <c r="L56" s="148">
         <f>IF($A56=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M56">
+      <c r="M56" s="149">
         <f>J56+L56</f>
         <v/>
       </c>
-      <c r="N56">
+      <c r="N56" s="149">
         <f>D56-M56</f>
         <v/>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="n">
+    <row r="57" ht="13" customHeight="1">
+      <c r="A57" s="147" t="n">
         <v>22</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="148">
         <f>IF(AND($A57&gt;=$C$8,$A57&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C57">
+      <c r="C57" s="148">
         <f>IF($A57=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D57">
+      <c r="D57" s="149">
         <f>B57+C57</f>
         <v/>
       </c>
-      <c r="E57">
+      <c r="E57" s="148">
         <f>IF($A57=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F57">
+      <c r="F57" s="148">
         <f>IF(AND($A57&gt;=1,$A57&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G57">
+      <c r="G57" s="148">
         <f>IF(AND($A57&gt;=$C$11,$A57&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H57">
+      <c r="H57" s="148">
         <f>IF(AND($A57&gt;=$C$8,$A57&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I57">
+      <c r="I57" s="148">
         <f>IF($A57=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J57">
+      <c r="J57" s="149">
         <f>E57+F57+G57+H57+I57</f>
         <v/>
       </c>
-      <c r="K57">
+      <c r="K57" s="149">
         <f>D57-J57</f>
         <v/>
       </c>
-      <c r="L57">
+      <c r="L57" s="148">
         <f>IF($A57=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M57">
+      <c r="M57" s="149">
         <f>J57+L57</f>
         <v/>
       </c>
-      <c r="N57">
+      <c r="N57" s="149">
         <f>D57-M57</f>
         <v/>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="n">
+    <row r="58" ht="13" customHeight="1">
+      <c r="A58" s="147" t="n">
         <v>23</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="153">
         <f>IF(AND($A58&gt;=$C$8,$A58&lt;=$C$9-1),$C$15*$C$10/($C$9-$C$8),0)</f>
         <v/>
       </c>
-      <c r="C58">
+      <c r="C58" s="153">
         <f>IF($A58=$C$9,$C$15*(1-$C$10),0)</f>
         <v/>
       </c>
-      <c r="D58">
+      <c r="D58" s="154">
         <f>B58+C58</f>
         <v/>
       </c>
-      <c r="E58">
+      <c r="E58" s="153">
         <f>IF($A58=0,$C$16,0)</f>
         <v/>
       </c>
-      <c r="F58">
+      <c r="F58" s="153">
         <f>IF(AND($A58&gt;=1,$A58&lt;=$C$7),$C$17/$C$7,0)</f>
         <v/>
       </c>
-      <c r="G58">
+      <c r="G58" s="153">
         <f>IF(AND($A58&gt;=$C$11,$A58&lt;=$C$12),$C$18/($C$12-$C$11+1),0)</f>
         <v/>
       </c>
-      <c r="H58">
+      <c r="H58" s="153">
         <f>IF(AND($A58&gt;=$C$8,$A58&lt;=$C$9),$C$19/($C$9-$C$8+1),0)</f>
         <v/>
       </c>
-      <c r="I58">
+      <c r="I58" s="153">
         <f>IF($A58=$C$9,$C$20,0)</f>
         <v/>
       </c>
-      <c r="J58">
+      <c r="J58" s="154">
         <f>E58+F58+G58+H58+I58</f>
         <v/>
       </c>
-      <c r="K58">
+      <c r="K58" s="154">
         <f>D58-J58</f>
         <v/>
       </c>
-      <c r="L58">
+      <c r="L58" s="153">
         <f>IF($A58=$C$9,$C$21,0)</f>
         <v/>
       </c>
-      <c r="M58">
+      <c r="M58" s="154">
         <f>J58+L58</f>
         <v/>
       </c>
-      <c r="N58">
+      <c r="N58" s="154">
         <f>D58-M58</f>
         <v/>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
+    <row r="59" ht="6" customHeight="1"/>
+    <row r="60" ht="6" customHeight="1"/>
+    <row r="61" ht="15" customHeight="1">
+      <c r="A61" s="139" t="inlineStr">
         <is>
           <t>RESULTADOS</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
+    <row r="62" ht="6" customHeight="1"/>
+    <row r="63" ht="15" customHeight="1">
+      <c r="A63" s="155" t="inlineStr">
         <is>
           <t>VAN Proyecto Puro (UF)</t>
         </is>
       </c>
-      <c r="C63">
+      <c r="C63" s="156">
         <f>K35+NPV(C4,K36:K58)</f>
         <v/>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+    <row r="64" ht="15" customHeight="1">
+      <c r="A64" s="155" t="inlineStr">
         <is>
           <t>VAN Proyecto Financiado (UF)</t>
         </is>
       </c>
-      <c r="C64">
+      <c r="C64" s="156">
         <f>N35+NPV(C4,N36:N58)</f>
         <v/>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
+    <row r="65" ht="6" customHeight="1"/>
+    <row r="66" ht="15" customHeight="1">
+      <c r="A66" s="135" t="inlineStr">
         <is>
           <t>TIR mensual Proyecto Puro</t>
         </is>
       </c>
-      <c r="C66">
+      <c r="C66" s="157">
         <f>IRR(K35:K58)</f>
         <v/>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
+    <row r="67" ht="15" customHeight="1">
+      <c r="A67" s="135" t="inlineStr">
         <is>
           <t>TIR mensual Proyecto Financiado</t>
         </is>
       </c>
-      <c r="C67">
+      <c r="C67" s="157">
         <f>IRR(N35:N58)</f>
         <v/>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
+    <row r="68" ht="6" customHeight="1"/>
+    <row r="69" ht="15" customHeight="1">
+      <c r="A69" s="155" t="inlineStr">
         <is>
           <t>TIR anual Proyecto Puro</t>
         </is>
       </c>
-      <c r="C69">
+      <c r="C69" s="158">
         <f>(1+IRR(K35:K58))^12-1</f>
         <v/>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
+    <row r="70" ht="15" customHeight="1">
+      <c r="A70" s="155" t="inlineStr">
         <is>
           <t>TIR anual Proyecto Financiado</t>
         </is>
       </c>
-      <c r="C70">
+      <c r="C70" s="158">
         <f>(1+IRR(N35:N58))^12-1</f>
         <v/>
       </c>
     </row>
+    <row r="71" ht="6" customHeight="1"/>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Nota: Los valores de TIR anual calculados arriba actualizan automáticamente las celdas B18 y B19 de la hoja "Resultados".</t>
+      <c r="A72" s="159" t="inlineStr">
+        <is>
+          <t>Nota: Los valores de TIR anual calculados arriba actualizan automáticamente las celdas D18 y D19 de la hoja "Resultados".</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="155" t="inlineStr">
+        <is>
+          <t>Leyenda:</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="13.5" customHeight="1">
+      <c r="A75" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Input (editable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="13.5" customHeight="1">
+      <c r="A76" s="161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Fórmula (calculada)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="13.5" customHeight="1">
+      <c r="A77" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Referencia cruzada (otra hoja)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A33:N33"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>